<commit_message>
Adição de vários métodos de extração. Tentativa de refatoração
</commit_message>
<xml_diff>
--- a/exports/resultados_cnj.xlsx
+++ b/exports/resultados_cnj.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,20 +436,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Subtítulo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Resultado</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
@@ -458,324 +463,608 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos) Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>1º Grau1º Grau</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>108,62%</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2025-11-27 17:45</t>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos) Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Turma RecursalTurma Recursal</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>104,28%</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2025-11-27 17:45</t>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:56</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos) Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Juizado EspecialJuizado Especial</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>101,10%</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2025-11-27 17:45</t>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:56</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos) Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+          <t>Meta 1: Julgar mais processos que os distribuídos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Julgar quantidade maior de processos de conhecimento do que os distribuídos de 20/12/24 a 19/12/25, excluídos os suspensos e sobrestados de 20/12/24 a 19/12/25.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>2º Grau2º Grau</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>93,29%</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2025-11-27 17:45</t>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:56</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos) Identificar e julgar até 31/12/2025: Superior Tribunal de Justiça: 100% dos processos distribuídos até 31/12/2018. Tribunal Superior do Trabalho: 100% dos processos distribuídos até 31/12/2019. Justiça Estadual: pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais. Justiça Federal: todos os processos distribuídos há 16 anos (2009), 85% dos processos distribuídos até 31/12/2021 no 1º e 2º grau e 100% dos processos distribuídos até 31/12/2022 nos Juizados Especiais Federais e nas Turmas Recursais. Justiça do Trabalho: pelo menos, 94% dos processos distribuídos até 31/12/2023, nos 1º e 2º graus e 100% dos processos pendentes de julgamento há 5 anos (2020) ou mais. Justiça Eleitoral: 70% dos processos distribuídos até 31/12/2023 e todos os processos de conhecimento pendentes de julgamento há 6 anos (2019) ou mais. Justiça Militar da União: todos os processos de conhecimento pendentes de julgamento há 5 anos (2020) ou mais e 95% dos processos distribuídos até 31/12/2022 nas Auditorias e 99% dos processos distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: todos os processos de conhecimento pendentes de julgamento há 3 anos (2022) ou mais e 90% dos processos distribuídos até 31/12/2023 nas Auditorias, e 95% dos processos distribuídos até 31/12/2024 no 2º grau.</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar até 31/12/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>1º Grau1º Grau</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>106,49%</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2025-11-27 17:45</t>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:56</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos) Identificar e julgar até 31/12/2025: Superior Tribunal de Justiça: 100% dos processos distribuídos até 31/12/2018. Tribunal Superior do Trabalho: 100% dos processos distribuídos até 31/12/2019. Justiça Estadual: pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais. Justiça Federal: todos os processos distribuídos há 16 anos (2009), 85% dos processos distribuídos até 31/12/2021 no 1º e 2º grau e 100% dos processos distribuídos até 31/12/2022 nos Juizados Especiais Federais e nas Turmas Recursais. Justiça do Trabalho: pelo menos, 94% dos processos distribuídos até 31/12/2023, nos 1º e 2º graus e 100% dos processos pendentes de julgamento há 5 anos (2020) ou mais. Justiça Eleitoral: 70% dos processos distribuídos até 31/12/2023 e todos os processos de conhecimento pendentes de julgamento há 6 anos (2019) ou mais. Justiça Militar da União: todos os processos de conhecimento pendentes de julgamento há 5 anos (2020) ou mais e 95% dos processos distribuídos até 31/12/2022 nas Auditorias e 99% dos processos distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: todos os processos de conhecimento pendentes de julgamento há 3 anos (2022) ou mais e 90% dos processos distribuídos até 31/12/2023 nas Auditorias, e 95% dos processos distribuídos até 31/12/2024 no 2º grau.</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar até 31/12/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>2º Grau2º Grau</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>108,61%</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2025-11-27 17:45</t>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:56</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos) Identificar e julgar até 31/12/2025: Superior Tribunal de Justiça: 100% dos processos distribuídos até 31/12/2018. Tribunal Superior do Trabalho: 100% dos processos distribuídos até 31/12/2019. Justiça Estadual: pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais. Justiça Federal: todos os processos distribuídos há 16 anos (2009), 85% dos processos distribuídos até 31/12/2021 no 1º e 2º grau e 100% dos processos distribuídos até 31/12/2022 nos Juizados Especiais Federais e nas Turmas Recursais. Justiça do Trabalho: pelo menos, 94% dos processos distribuídos até 31/12/2023, nos 1º e 2º graus e 100% dos processos pendentes de julgamento há 5 anos (2020) ou mais. Justiça Eleitoral: 70% dos processos distribuídos até 31/12/2023 e todos os processos de conhecimento pendentes de julgamento há 6 anos (2019) ou mais. Justiça Militar da União: todos os processos de conhecimento pendentes de julgamento há 5 anos (2020) ou mais e 95% dos processos distribuídos até 31/12/2022 nas Auditorias e 99% dos processos distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: todos os processos de conhecimento pendentes de julgamento há 3 anos (2022) ou mais e 90% dos processos distribuídos até 31/12/2023 nas Auditorias, e 95% dos processos distribuídos até 31/12/2024 no 2º grau.</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar até 31/12/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Juizado EspecialJuizado Especial</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>98,04%</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2025-11-27 17:45</t>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:56</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos) Identificar e julgar até 31/12/2025: Superior Tribunal de Justiça: 100% dos processos distribuídos até 31/12/2018. Tribunal Superior do Trabalho: 100% dos processos distribuídos até 31/12/2019. Justiça Estadual: pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais. Justiça Federal: todos os processos distribuídos há 16 anos (2009), 85% dos processos distribuídos até 31/12/2021 no 1º e 2º grau e 100% dos processos distribuídos até 31/12/2022 nos Juizados Especiais Federais e nas Turmas Recursais. Justiça do Trabalho: pelo menos, 94% dos processos distribuídos até 31/12/2023, nos 1º e 2º graus e 100% dos processos pendentes de julgamento há 5 anos (2020) ou mais. Justiça Eleitoral: 70% dos processos distribuídos até 31/12/2023 e todos os processos de conhecimento pendentes de julgamento há 6 anos (2019) ou mais. Justiça Militar da União: todos os processos de conhecimento pendentes de julgamento há 5 anos (2020) ou mais e 95% dos processos distribuídos até 31/12/2022 nas Auditorias e 99% dos processos distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: todos os processos de conhecimento pendentes de julgamento há 3 anos (2022) ou mais e 90% dos processos distribuídos até 31/12/2023 nas Auditorias, e 95% dos processos distribuídos até 31/12/2024 no 2º grau.</t>
+          <t>Meta 2 – Julgar processos mais antigos (todos os segmentos)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>Identificar e julgar até 31/12/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>pelo menos, 80% dos processos distribuídos até 31/12/2021 no 1º grau, 90% dos processos distribuídos até 31/12/2022 no 2º grau, 95% dos processos distribuídos até 31/12/2022 nos Juizados Especiais e Turmas Recursais e 100% dos processos de conhecimento pendentes de julgamento há 15 anos (2010) ou mais.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>Turma RecursalTurma Recursal</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>100,77%</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2025-11-27 17:45</t>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:56</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Meta 3 – Estimular a conciliação Justiça Estadual: Aumentar o indicador Índice de Conciliação do Justiça em Números em 1 ponto percentual em relação a 2024. Cláusula de barreira: 17% de Índice de Conciliação. Justiça Federal: Aumentar o Índice de Conciliação do Justiça em Números em 0,5 ponto percentual em relação ao biênio 2023/2024. Cláusula de barreira: 8% de Índice de Conciliação. Justiça do Trabalho: Aumentar o índice de conciliação em 0,5 ponto percentual em relação à média do biênio 2022/2023 ou alcançar, no mínimo, 38% de conciliação.</t>
+          <t>Meta 3 – Estimular a conciliação</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Aumentar o indicador Índice de Conciliação do Justiça em Números em 1 ponto percentual em relação a 2024. Cláusula de barreira: 17% de Índice de Conciliação.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>100,00%</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2025-11-27 17:46</t>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:56</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais Superior Tribunal de Justiça: Identificar e julgar até 31/12/2025, 90% das ações de improbidade administrativa e das ações penais relacionadas aos crimes contra a Administração Pública distribuídas até 31/12/2023 e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Estadual: Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Federal: Identificar e julgar até 31/12/2025, 70% das ações de improbidade administrativa e das ações penais relacionadas aos crimes contra a administração pública distribuídas até 31/12/2022 e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Eleitoral: Identificar e julgar até 31/12/2025, 90% dos processos referentes às eleições de 2022 e 50% dos processos referentes às eleições de 2024, distribuídos até 31/12/2024, que possam importar na perda de mandato eletivo ou em inelegibilidade.  Justiça Militar da União: Identificar e julgar até 31/12/2025, 95% dos processos da meta distribuídos até 31/12/2022 nas Auditorias e 99% dos processos da meta distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: Identificar e julgar até 31/12/2025, 95% das ações penais relacionadas aos crimes contra a Administração Pública, abrangendo, inclusive, a Lei 13.491/17, distribuídas até 31/12/2023 no 1º grau, e pelo menos 95% das distribuídas no 2º grau até 31/12/2024.</t>
+          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>Total Real</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>140,04%</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2025-11-27 17:46</t>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:56</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais Superior Tribunal de Justiça: Identificar e julgar até 31/12/2025, 90% das ações de improbidade administrativa e das ações penais relacionadas aos crimes contra a Administração Pública distribuídas até 31/12/2023 e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Estadual: Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Federal: Identificar e julgar até 31/12/2025, 70% das ações de improbidade administrativa e das ações penais relacionadas aos crimes contra a administração pública distribuídas até 31/12/2022 e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021. Justiça Eleitoral: Identificar e julgar até 31/12/2025, 90% dos processos referentes às eleições de 2022 e 50% dos processos referentes às eleições de 2024, distribuídos até 31/12/2024, que possam importar na perda de mandato eletivo ou em inelegibilidade.  Justiça Militar da União: Identificar e julgar até 31/12/2025, 95% dos processos da meta distribuídos até 31/12/2022 nas Auditorias e 99% dos processos da meta distribuídos até 31/12/2023 no STM. Justiça Militar Estadual: Identificar e julgar até 31/12/2025, 95% das ações penais relacionadas aos crimes contra a Administração Pública, abrangendo, inclusive, a Lei 13.491/17, distribuídas até 31/12/2023 no 1º grau, e pelo menos 95% das distribuídas no 2º grau até 31/12/2024.</t>
+          <t>Meta 4 – Priorizar o julgamento dos processos relativos aos crimes contra a Administração Pública, à improbidade administrativa e aos ilícitos eleitorais</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>Identificar e julgar até 31/12/2025, 65% das ações de improbidade administrativa e das ações penais relacionadas a crimes contra a Administração Pública, distribuídas até 31/12/2021, em especial as relativas a corrupção ativa e passiva, peculato em geral e concussão e identificar e julgar até 26/10/2025, 100% das ações de improbidade administrativa distribuídas até 26/10/2021.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>Total Submeta</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>73,19%</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2025-11-27 17:46</t>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:56</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Meta 5 – Reduzir a taxa de congestionamento Superior Tribunal de Justiça: Reduzir em 0,5 ponto percentual, até 31/12/2025, a taxa de congestionamento dos processos no Superior Tribunal de Justiça, referente ao apurado em 2024. Tribunal Superior do Trabalho: Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida, exceto execuções fiscais, em relação a 2024.  Justiça Federal: Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida, exceto execuções fiscais, em relação a 2024. Cláusula de barreira: 43%. Justiça do Trabalho: Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida, exceto execuções fiscais, em relação a 2024. Cláusula de barreira na fase de conhecimento: 40%. Cláusula de barreira na fase de execução: 65%. Justiça Estadual: Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida de processo de conhecimento, em relação a 2024. Cláusula de barreira: 56%. Justiça Militar da União: Reduzir, no mínimo, em 0,5 ponto percentual a taxa de congestionamento líquida na fase de conhecimento no 1º grau, em relação a 2024. Justiça Militar Estadual: Reduzir, no mínimo, em 0,5 ponto percentual a taxa de congestionamento líquida na fase de conhecimento no 1º grau, em relação a 2023.</t>
+          <t>Meta 5 – Reduzir a taxa de congestionamento</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Filtrar por:</t>
+          <t>N/D</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>Reduzir em 0,5 ponto percentual a taxa de congestionamento líquida de processo de conhecimento, em relação a 2024. Cláusula de barreira: 56%.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>92,30%</t>
-        </is>
-      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025-11-27 17:46</t>
+          <t>88,83%</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Meta 6 – Priorizar o julgamento das ações ambientais</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Identificar e julgar até 31/12/2025</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>50% dos processos relacionados às ações ambientais distribuídos até 31/12/2024.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>84,76%</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Meta 7 – Priorizar o julgamento dos processos relacionados aos indígenas e quilombolas</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Identificar e julgar até 31/12/2025</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>50% dos processos relacionados aos direitos das comunidades indígenas e 50% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Total Indígenas</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>120,00%</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Meta 7 – Priorizar o julgamento dos processos relacionados aos indígenas e quilombolas</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Identificar e julgar até 31/12/2025</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>50% dos processos relacionados aos direitos das comunidades indígenas e 50% dos processos relacionados aos direitos das comunidades quilombolas distribuídos até 31/12/2024.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Total Quilombola</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>100,00%</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Identificar e julgar, até 31/12/2025</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Total Violência Doméstica</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>91,31%</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Meta 8 – Priorizar o julgamento dos processos relacionados ao feminicídio e à violência doméstica e familiar contra as mulheres</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Identificar e julgar, até 31/12/2025</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>75% dos casos de feminicídio distribuídos até 31/12/2023 e 90% dos casos de violência doméstica e familiar contra a mulher distribuídos até 31/12/2023.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Total Feminicídio</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>108,62%</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Meta 10 – Promover os direitos da criança e do adolescente.</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Identificar e julgar, até 31/12/2025, no 1º grau, 90% e no 2º grau, 100% dos processos em fase de conhecimento, nas competências da Infância e Juventude cível e de apuração de ato infracional, distribuídos até 31/12/2023 nas respectivas instâncias.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Total 1º Grau</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>86,57%</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Meta 10 – Promover os direitos da criança e do adolescente.</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Identificar e julgar, até 31/12/2025, no 1º grau, 90% e no 2º grau, 100% dos processos em fase de conhecimento, nas competências da Infância e Juventude cível e de apuração de ato infracional, distribuídos até 31/12/2023 nas respectivas instâncias.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Total 2º Grau</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>85,09%</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2025-12-02 15:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizações da extração do Jira e inclusão da Meta 9 na extração do CNJ
</commit_message>
<xml_diff>
--- a/exports/resultados_cnj.xlsx
+++ b/exports/resultados_cnj.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,17 +478,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1º Grau</t>
+          <t>Turma Recursal</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>108,62%</t>
+          <t>106,30%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2025-12-03 16:27</t>
+          <t>2026-02-05 15:46</t>
         </is>
       </c>
     </row>
@@ -510,17 +510,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Turma Recursal</t>
+          <t>1º Grau</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>104,28%</t>
+          <t>96,76%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025-12-03 16:27</t>
+          <t>2026-02-05 15:46</t>
         </is>
       </c>
     </row>
@@ -542,17 +542,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Juizado Especial</t>
+          <t>2º Grau</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>101,10%</t>
+          <t>93,31%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025-12-03 16:27</t>
+          <t>2026-02-05 15:46</t>
         </is>
       </c>
     </row>
@@ -574,17 +574,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2º Grau</t>
+          <t>Juizado Especial</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>93,29%</t>
+          <t>92,97%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2025-12-03 16:27</t>
+          <t>2026-02-05 15:46</t>
         </is>
       </c>
     </row>
@@ -611,12 +611,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>103,05%</t>
+          <t>95,65%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2025-12-03 16:27</t>
+          <t>2026-02-05 15:46</t>
         </is>
       </c>
     </row>
@@ -643,12 +643,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>106,49%</t>
+          <t>107,06%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2025-12-03 16:27</t>
+          <t>2026-02-05 15:46</t>
         </is>
       </c>
     </row>
@@ -675,12 +675,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>108,61%</t>
+          <t>109,38%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2025-12-03 16:27</t>
+          <t>2026-02-05 15:46</t>
         </is>
       </c>
     </row>
@@ -707,12 +707,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>98,29%</t>
+          <t>99,52%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2025-12-03 16:27</t>
+          <t>2026-02-05 15:46</t>
         </is>
       </c>
     </row>
@@ -739,12 +739,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>44,66%</t>
+          <t>48,99%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2025-12-03 16:27</t>
+          <t>2026-02-05 15:46</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2025-12-03 16:27</t>
+          <t>2026-02-05 15:47</t>
         </is>
       </c>
     </row>
@@ -803,12 +803,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>140,04%</t>
+          <t>142,82%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2025-12-03 16:28</t>
+          <t>2026-02-05 15:47</t>
         </is>
       </c>
     </row>
@@ -835,12 +835,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>73,19%</t>
+          <t>73,18%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2025-12-03 16:28</t>
+          <t>2026-02-05 15:47</t>
         </is>
       </c>
     </row>
@@ -867,12 +867,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>88,83%</t>
+          <t>83,53%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2025-12-03 16:28</t>
+          <t>2026-02-05 15:47</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>84,76%</t>
+          <t>90,88%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2025-12-03 16:28</t>
+          <t>2026-02-05 15:47</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2025-12-03 16:28</t>
+          <t>2026-02-05 15:47</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2025-12-03 16:28</t>
+          <t>2026-02-05 15:47</t>
         </is>
       </c>
     </row>
@@ -995,12 +995,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>91,31%</t>
+          <t>92,01%</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2025-12-03 16:29</t>
+          <t>2026-02-05 15:48</t>
         </is>
       </c>
     </row>
@@ -1027,19 +1027,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>108,62%</t>
+          <t>109,71%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2025-12-03 16:29</t>
+          <t>2026-02-05 15:48</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Meta 10 – Promover os direitos da criança e do adolescente.</t>
+          <t>Meta 9 – Estimular a inovação no Poder Judiciário</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1049,22 +1049,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Identificar e julgar, até 31/12/2025, no 1º grau, 90% e no 2º grau, 100% dos processos em fase de conhecimento, nas competências da Infância e Juventude cível e de apuração de ato infracional, distribuídos até 31/12/2023 nas respectivas instâncias.</t>
+          <t>Desenvolver, no ano de 2025, dois projetos relacionados à Agenda 2030 da ONU, oriundos do Laboratório de Inovação, com participação de pelo menos um laboratório de outra instituição pública, e que gerem benefícios à sociedade.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1º Grau</t>
+          <t>Total Meta 9</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>86,57%</t>
+          <t>100,00%</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2025-12-03 16:29</t>
+          <t>2026-02-05 15:48</t>
         </is>
       </c>
     </row>
@@ -1086,17 +1086,49 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
+          <t>1º Grau</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>87,43%</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-02-05 15:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Meta 10 – Promover os direitos da criança e do adolescente.</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Identificar e julgar, até 31/12/2025, no 1º grau, 90% e no 2º grau, 100% dos processos em fase de conhecimento, nas competências da Infância e Juventude cível e de apuração de ato infracional, distribuídos até 31/12/2023 nas respectivas instâncias.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>2º Grau</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>85,09%</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>2025-12-03 16:29</t>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>85,17%</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-02-05 15:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização da extração anual do extrator unico
</commit_message>
<xml_diff>
--- a/exports/resultados_cnj.xlsx
+++ b/exports/resultados_cnj.xlsx
@@ -488,7 +488,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-02-05 15:46</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-05 15:46</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-02-05 15:46</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-02-05 15:46</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-02-05 15:46</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-02-05 15:46</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-02-05 15:46</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-02-05 15:46</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-02-05 15:46</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-02-05 15:47</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-02-05 15:47</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-02-05 15:47</t>
+          <t>2026-02-11 09:41</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-02-05 15:47</t>
+          <t>2026-02-11 09:42</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-02-05 15:47</t>
+          <t>2026-02-11 09:42</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-02-05 15:47</t>
+          <t>2026-02-11 09:42</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-02-05 15:47</t>
+          <t>2026-02-11 09:42</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-02-05 15:48</t>
+          <t>2026-02-11 09:42</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-02-05 15:48</t>
+          <t>2026-02-11 09:42</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-02-05 15:48</t>
+          <t>2026-02-11 09:42</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-02-05 15:48</t>
+          <t>2026-02-11 09:43</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-02-05 15:48</t>
+          <t>2026-02-11 09:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajuste na extração do Jira, ajustes CSS feitos
</commit_message>
<xml_diff>
--- a/exports/resultados_cnj.xlsx
+++ b/exports/resultados_cnj.xlsx
@@ -483,12 +483,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>106,30%</t>
+          <t>105,05%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:19</t>
         </is>
       </c>
     </row>
@@ -515,12 +515,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>96,76%</t>
+          <t>97,24%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:19</t>
         </is>
       </c>
     </row>
@@ -547,12 +547,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>93,31%</t>
+          <t>92,85%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:19</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>92,97%</t>
+          <t>92,80%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:19</t>
         </is>
       </c>
     </row>
@@ -611,12 +611,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>95,65%</t>
+          <t>95,66%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:19</t>
         </is>
       </c>
     </row>
@@ -643,12 +643,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>107,06%</t>
+          <t>107,43%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:19</t>
         </is>
       </c>
     </row>
@@ -675,12 +675,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>109,38%</t>
+          <t>109,35%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:19</t>
         </is>
       </c>
     </row>
@@ -707,12 +707,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>99,52%</t>
+          <t>99,73%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:19</t>
         </is>
       </c>
     </row>
@@ -739,12 +739,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>48,99%</t>
+          <t>50,10%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:19</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:20</t>
         </is>
       </c>
     </row>
@@ -803,12 +803,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>142,82%</t>
+          <t>143,25%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:20</t>
         </is>
       </c>
     </row>
@@ -835,12 +835,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>73,18%</t>
+          <t>73,23%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-02-11 09:41</t>
+          <t>2026-02-27 18:20</t>
         </is>
       </c>
     </row>
@@ -867,12 +867,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>83,53%</t>
+          <t>85,34%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-02-11 09:42</t>
+          <t>2026-02-27 18:20</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>90,88%</t>
+          <t>94,00%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-02-11 09:42</t>
+          <t>2026-02-27 18:20</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-02-11 09:42</t>
+          <t>2026-02-27 18:21</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-02-11 09:42</t>
+          <t>2026-02-27 18:21</t>
         </is>
       </c>
     </row>
@@ -995,12 +995,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>92,01%</t>
+          <t>92,88%</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-02-11 09:42</t>
+          <t>2026-02-27 18:21</t>
         </is>
       </c>
     </row>
@@ -1027,12 +1027,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>109,71%</t>
+          <t>110,94%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-02-11 09:42</t>
+          <t>2026-02-27 18:21</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-02-11 09:42</t>
+          <t>2026-02-27 18:21</t>
         </is>
       </c>
     </row>
@@ -1091,12 +1091,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>87,43%</t>
+          <t>88,27%</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-02-11 09:43</t>
+          <t>2026-02-27 18:21</t>
         </is>
       </c>
     </row>
@@ -1123,12 +1123,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>85,17%</t>
+          <t>85,18%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-02-11 09:43</t>
+          <t>2026-02-27 18:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizações no projeto em conferência
</commit_message>
<xml_diff>
--- a/exports/resultados_cnj.xlsx
+++ b/exports/resultados_cnj.xlsx
@@ -488,7 +488,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-03-02 10:21</t>
+          <t>2026-03-03 10:06</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-03-02 10:21</t>
+          <t>2026-03-03 10:06</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-03-02 10:21</t>
+          <t>2026-03-03 10:06</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-03-02 10:21</t>
+          <t>2026-03-03 10:06</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-03-02 10:21</t>
+          <t>2026-03-03 10:06</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-03-02 10:22</t>
+          <t>2026-03-03 10:06</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-03-02 10:22</t>
+          <t>2026-03-03 10:06</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-03-02 10:22</t>
+          <t>2026-03-03 10:06</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-03-02 10:22</t>
+          <t>2026-03-03 10:06</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-03-02 10:22</t>
+          <t>2026-03-03 10:07</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-03-02 10:22</t>
+          <t>2026-03-03 10:07</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-03-02 10:22</t>
+          <t>2026-03-03 10:07</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-03-02 10:22</t>
+          <t>2026-03-03 10:07</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-03-02 10:22</t>
+          <t>2026-03-03 10:07</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-03-02 10:23</t>
+          <t>2026-03-03 10:08</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-03-02 10:23</t>
+          <t>2026-03-03 10:08</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-03-02 10:23</t>
+          <t>2026-03-03 10:08</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-03-02 10:23</t>
+          <t>2026-03-03 10:08</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-03-02 10:23</t>
+          <t>2026-03-03 10:08</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-03-02 10:23</t>
+          <t>2026-03-03 10:08</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-03-02 10:23</t>
+          <t>2026-03-03 10:08</t>
         </is>
       </c>
     </row>

</xml_diff>